<commit_message>
Asp 5638 cherry pick fixed to next release (#2796)
* For No Stock Report:
- Corrected parameters order
- Corrected default in dates
- Applying date filter to day instead of createdOn
- Change order of joins to show correct quantities
- Remove filter by PartnerConsumable

* Format fixes y report template

---------

Co-authored-by: nsabaj95 <nsabaj@hotmail.com>
</commit_message>
<xml_diff>
--- a/api/templates/no_stock/en.xlsx
+++ b/api/templates/no_stock/en.xlsx
@@ -1,37 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\no_stock\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\no_stock\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDA49C7B-E617-47A0-AC41-E384D78A2BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16920" tabRatio="815"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NoStock" sheetId="6" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
-      <mx:ArchID Flags="2"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
-    <t>Devices with maintanance status set to No-Stock</t>
-  </si>
-  <si>
-    <t>* Days set to No-Stock represent the days between a device was manually marked out of stock and then changed it's status again</t>
-  </si>
-  <si>
     <t>Device</t>
   </si>
   <si>
@@ -66,22 +56,20 @@
   </si>
   <si>
     <t>&lt;SitesLabel&gt;: &lt;Sites&gt;</t>
+  </si>
+  <si>
+    <t>Devices with maintenance status set to No-Stock</t>
+  </si>
+  <si>
+    <t>* Days set to No-Stock represent the days between a device was manually marked out of stock and then changed it status again</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -113,6 +101,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -123,12 +125,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FF3CC0DD"/>
+        <bgColor rgb="FF00CCFF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -165,13 +167,15 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="medium">
-        <color auto="1"/>
+      <right style="thin">
+        <color indexed="64"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -181,149 +185,82 @@
       <left style="medium">
         <color auto="1"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
+      <right style="medium">
         <color auto="1"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="43">
+  <cellStyleXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="43" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="43" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="43">
+  <cellStyles count="45">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -367,6 +304,8 @@
     <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="43" xr:uid="{5BFB2D89-4F64-4525-B509-B4EB88CBBC59}"/>
+    <cellStyle name="Percent 2" xfId="44" xr:uid="{1E23EC80-D07A-46B9-BE91-C02959573C6E}"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -393,7 +332,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -730,86 +669,85 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.296875" customWidth="1"/>
     <col min="2" max="2" width="20" style="3" customWidth="1"/>
-    <col min="3" max="3" width="11.19921875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="21.8984375" style="3" customWidth="1"/>
     <col min="4" max="4" width="14.3984375" customWidth="1"/>
     <col min="6" max="6" width="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="5">
+        <v>5</v>
+      </c>
+      <c r="B10" s="4">
         <v>2</v>
       </c>
-      <c r="C10" s="4"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+    </row>
+    <row r="11" spans="1:3" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="12"/>
+    </row>
+    <row r="12" spans="1:3" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>6</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>